<commit_message>
feat(internacional): antecedente de KR, TW y ON, visor HTML y revisión experta
- Secundaria baja de KR (중학교), TW (第四學習階段) y ON (SNC1W 2022) como antecedente:
  438 objetivos que fechan la primera aparición sin entrar al núcleo de 9.°–11.°.
- Excepción de especialización con núcleo «sólido» (principal en un objetivo o
  secundario en dos); 5 clases corregidas en revisiones.json con evidencia citada.
- Normalización de ids sin asignatura solo si el resultado es único en el catálogo.
- internacional/visor.html: pestañas por asignatura, filtros por clase y evidencia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/Contraste_fisica.xlsx
+++ b/internacional/Contraste_fisica.xlsx
@@ -765,7 +765,7 @@
         <v>9.5</v>
       </c>
       <c r="M5" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O5" t="n">
         <v>1</v>
@@ -836,6 +836,9 @@
       <c r="L6" t="n">
         <v>9.5</v>
       </c>
+      <c r="M6" t="n">
+        <v>7</v>
+      </c>
       <c r="O6" t="n">
         <v>1</v>
       </c>
@@ -1232,9 +1235,15 @@
       <c r="F13" t="n">
         <v>8</v>
       </c>
+      <c r="J13" t="n">
+        <v>7</v>
+      </c>
       <c r="K13" t="n">
         <v>9</v>
       </c>
+      <c r="M13" t="n">
+        <v>7</v>
+      </c>
       <c r="O13" t="n">
         <v>1</v>
       </c>
@@ -1268,9 +1277,15 @@
       <c r="G14" t="n">
         <v>6</v>
       </c>
+      <c r="J14" t="n">
+        <v>7</v>
+      </c>
       <c r="K14" t="n">
         <v>9</v>
       </c>
+      <c r="M14" t="n">
+        <v>7</v>
+      </c>
       <c r="T14" t="n">
         <v>1</v>
       </c>
@@ -1361,11 +1376,14 @@
       <c r="I16" t="n">
         <v>9.5</v>
       </c>
+      <c r="J16" t="n">
+        <v>7</v>
+      </c>
       <c r="L16" t="n">
         <v>9.5</v>
       </c>
       <c r="M16" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O16" t="n">
         <v>1</v>
@@ -1481,9 +1499,15 @@
       <c r="I18" t="n">
         <v>7</v>
       </c>
+      <c r="J18" t="n">
+        <v>7</v>
+      </c>
       <c r="L18" t="n">
         <v>9.5</v>
       </c>
+      <c r="M18" t="n">
+        <v>7</v>
+      </c>
       <c r="O18" t="n">
         <v>1</v>
       </c>
@@ -1601,12 +1625,18 @@
       <c r="I20" t="n">
         <v>6</v>
       </c>
+      <c r="J20" t="n">
+        <v>7</v>
+      </c>
       <c r="K20" t="n">
         <v>9</v>
       </c>
       <c r="L20" t="n">
         <v>9.5</v>
       </c>
+      <c r="M20" t="n">
+        <v>7</v>
+      </c>
       <c r="O20" t="n">
         <v>1</v>
       </c>
@@ -1652,11 +1682,14 @@
       <c r="F21" t="n">
         <v>8</v>
       </c>
+      <c r="J21" t="n">
+        <v>7</v>
+      </c>
       <c r="L21" t="n">
         <v>9.5</v>
       </c>
       <c r="M21" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O21" t="n">
         <v>1</v>
@@ -1718,9 +1751,18 @@
       <c r="I22" t="n">
         <v>7</v>
       </c>
+      <c r="J22" t="n">
+        <v>7</v>
+      </c>
+      <c r="K22" t="n">
+        <v>8</v>
+      </c>
       <c r="L22" t="n">
         <v>9.5</v>
       </c>
+      <c r="M22" t="n">
+        <v>7</v>
+      </c>
       <c r="O22" t="n">
         <v>1</v>
       </c>
@@ -1931,6 +1973,9 @@
       <c r="K26" t="n">
         <v>9</v>
       </c>
+      <c r="M26" t="n">
+        <v>7</v>
+      </c>
       <c r="O26" t="n">
         <v>1</v>
       </c>
@@ -2241,7 +2286,7 @@
         <v>9.5</v>
       </c>
       <c r="M31" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="P31" t="n">
         <v>1</v>
@@ -2297,6 +2342,9 @@
       <c r="G32" t="n">
         <v>8.5</v>
       </c>
+      <c r="M32" t="n">
+        <v>7</v>
+      </c>
       <c r="O32" t="n">
         <v>1</v>
       </c>
@@ -2403,7 +2451,7 @@
         <v>9.5</v>
       </c>
       <c r="J34" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L34" t="n">
         <v>11</v>
@@ -2531,6 +2579,9 @@
       <c r="I36" t="n">
         <v>9.5</v>
       </c>
+      <c r="J36" t="n">
+        <v>7</v>
+      </c>
       <c r="M36" t="n">
         <v>9.5</v>
       </c>
@@ -2607,7 +2658,7 @@
         <v>9.5</v>
       </c>
       <c r="M37" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="N37" t="n">
         <v>1</v>
@@ -2675,11 +2726,14 @@
       <c r="I38" t="n">
         <v>5</v>
       </c>
+      <c r="J38" t="n">
+        <v>7</v>
+      </c>
       <c r="L38" t="n">
         <v>9.5</v>
       </c>
       <c r="M38" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O38" t="n">
         <v>1</v>
@@ -2759,6 +2813,9 @@
       <c r="L40" t="n">
         <v>9.5</v>
       </c>
+      <c r="M40" t="n">
+        <v>7</v>
+      </c>
       <c r="P40" t="n">
         <v>1</v>
       </c>
@@ -2801,6 +2858,9 @@
       <c r="I41" t="n">
         <v>2</v>
       </c>
+      <c r="J41" t="n">
+        <v>7</v>
+      </c>
       <c r="L41" t="n">
         <v>9.5</v>
       </c>
@@ -2856,11 +2916,14 @@
         <v>9.5</v>
       </c>
       <c r="J42" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L42" t="n">
         <v>9.5</v>
       </c>
+      <c r="M42" t="n">
+        <v>7</v>
+      </c>
       <c r="O42" t="n">
         <v>1</v>
       </c>
@@ -2918,6 +2981,9 @@
       <c r="L43" t="n">
         <v>11</v>
       </c>
+      <c r="M43" t="n">
+        <v>7</v>
+      </c>
       <c r="O43" t="n">
         <v>1</v>
       </c>
@@ -2973,7 +3039,7 @@
         <v>9.5</v>
       </c>
       <c r="J44" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L44" t="n">
         <v>9.5</v>
@@ -3044,9 +3110,15 @@
       <c r="I45" t="n">
         <v>2</v>
       </c>
+      <c r="J45" t="n">
+        <v>7</v>
+      </c>
       <c r="L45" t="n">
         <v>9.5</v>
       </c>
+      <c r="M45" t="n">
+        <v>7</v>
+      </c>
       <c r="O45" t="n">
         <v>1</v>
       </c>
@@ -3098,11 +3170,14 @@
       <c r="I46" t="n">
         <v>9.5</v>
       </c>
+      <c r="J46" t="n">
+        <v>7</v>
+      </c>
       <c r="L46" t="n">
         <v>9.5</v>
       </c>
       <c r="M46" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O46" t="n">
         <v>1</v>
@@ -3161,11 +3236,14 @@
       <c r="I47" t="n">
         <v>3</v>
       </c>
+      <c r="J47" t="n">
+        <v>7</v>
+      </c>
       <c r="L47" t="n">
         <v>9.5</v>
       </c>
       <c r="M47" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O47" t="n">
         <v>1</v>
@@ -3234,13 +3312,13 @@
         <v>7</v>
       </c>
       <c r="J48" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L48" t="n">
         <v>9.5</v>
       </c>
       <c r="M48" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O48" t="n">
         <v>1</v>
@@ -3308,6 +3386,12 @@
       <c r="G49" t="n">
         <v>8.5</v>
       </c>
+      <c r="J49" t="n">
+        <v>7</v>
+      </c>
+      <c r="M49" t="n">
+        <v>7</v>
+      </c>
       <c r="O49" t="n">
         <v>1</v>
       </c>
@@ -3359,11 +3443,17 @@
       <c r="I50" t="n">
         <v>7</v>
       </c>
+      <c r="J50" t="n">
+        <v>7</v>
+      </c>
+      <c r="K50" t="n">
+        <v>8</v>
+      </c>
       <c r="L50" t="n">
         <v>9.5</v>
       </c>
       <c r="M50" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O50" t="n">
         <v>1</v>
@@ -3428,9 +3518,18 @@
       <c r="I51" t="n">
         <v>2</v>
       </c>
+      <c r="J51" t="n">
+        <v>7</v>
+      </c>
+      <c r="K51" t="n">
+        <v>8</v>
+      </c>
       <c r="L51" t="n">
         <v>9.5</v>
       </c>
+      <c r="M51" t="n">
+        <v>7</v>
+      </c>
       <c r="O51" t="n">
         <v>1</v>
       </c>
@@ -3488,6 +3587,12 @@
       <c r="I52" t="n">
         <v>3</v>
       </c>
+      <c r="J52" t="n">
+        <v>7</v>
+      </c>
+      <c r="K52" t="n">
+        <v>8</v>
+      </c>
       <c r="L52" t="n">
         <v>9.5</v>
       </c>
@@ -3603,11 +3708,14 @@
         <v>6</v>
       </c>
       <c r="J54" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K54" t="n">
         <v>9</v>
       </c>
+      <c r="M54" t="n">
+        <v>7</v>
+      </c>
       <c r="O54" t="n">
         <v>1</v>
       </c>
@@ -3660,11 +3768,17 @@
         <v>2</v>
       </c>
       <c r="J55" t="n">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="K55" t="n">
+        <v>8</v>
       </c>
       <c r="L55" t="n">
         <v>9.5</v>
       </c>
+      <c r="M55" t="n">
+        <v>7</v>
+      </c>
       <c r="O55" t="n">
         <v>1</v>
       </c>
@@ -3719,9 +3833,15 @@
       <c r="I56" t="n">
         <v>8</v>
       </c>
+      <c r="J56" t="n">
+        <v>7</v>
+      </c>
       <c r="L56" t="n">
         <v>9.5</v>
       </c>
+      <c r="M56" t="n">
+        <v>7</v>
+      </c>
       <c r="O56" t="n">
         <v>1</v>
       </c>
@@ -3842,11 +3962,17 @@
       <c r="I58" t="n">
         <v>3</v>
       </c>
+      <c r="J58" t="n">
+        <v>7</v>
+      </c>
+      <c r="K58" t="n">
+        <v>8</v>
+      </c>
       <c r="L58" t="n">
         <v>9.5</v>
       </c>
       <c r="M58" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O58" t="n">
         <v>1</v>
@@ -3915,7 +4041,10 @@
         <v>10</v>
       </c>
       <c r="J59" t="n">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="K59" t="n">
+        <v>8</v>
       </c>
       <c r="M59" t="n">
         <v>9.5</v>
@@ -3986,9 +4115,15 @@
       <c r="I60" t="n">
         <v>2</v>
       </c>
+      <c r="J60" t="n">
+        <v>7</v>
+      </c>
       <c r="L60" t="n">
         <v>9.5</v>
       </c>
+      <c r="M60" t="n">
+        <v>7</v>
+      </c>
       <c r="O60" t="n">
         <v>1</v>
       </c>
@@ -4034,9 +4169,15 @@
       <c r="I61" t="n">
         <v>3</v>
       </c>
+      <c r="J61" t="n">
+        <v>7</v>
+      </c>
       <c r="L61" t="n">
         <v>9.5</v>
       </c>
+      <c r="M61" t="n">
+        <v>7</v>
+      </c>
       <c r="O61" t="n">
         <v>1</v>
       </c>
@@ -4098,13 +4239,16 @@
         <v>8</v>
       </c>
       <c r="J63" t="n">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="K63" t="n">
+        <v>8</v>
       </c>
       <c r="L63" t="n">
         <v>9.5</v>
       </c>
       <c r="M63" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O63" t="n">
         <v>1</v>
@@ -4169,9 +4313,15 @@
       <c r="I64" t="n">
         <v>4</v>
       </c>
+      <c r="J64" t="n">
+        <v>7</v>
+      </c>
       <c r="L64" t="n">
         <v>9.5</v>
       </c>
+      <c r="M64" t="n">
+        <v>7</v>
+      </c>
       <c r="O64" t="n">
         <v>1</v>
       </c>
@@ -4236,13 +4386,13 @@
         <v>8</v>
       </c>
       <c r="J65" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L65" t="n">
         <v>9.5</v>
       </c>
       <c r="M65" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="P65" t="n">
         <v>1</v>
@@ -4310,9 +4460,15 @@
       <c r="I66" t="n">
         <v>8</v>
       </c>
+      <c r="J66" t="n">
+        <v>7</v>
+      </c>
       <c r="L66" t="n">
         <v>9.5</v>
       </c>
+      <c r="M66" t="n">
+        <v>7</v>
+      </c>
       <c r="P66" t="n">
         <v>1</v>
       </c>
@@ -4370,11 +4526,14 @@
       <c r="G67" t="n">
         <v>6</v>
       </c>
+      <c r="J67" t="n">
+        <v>7</v>
+      </c>
       <c r="L67" t="n">
         <v>9.5</v>
       </c>
       <c r="M67" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O67" t="n">
         <v>1</v>
@@ -4427,9 +4586,15 @@
       <c r="I68" t="n">
         <v>6</v>
       </c>
+      <c r="J68" t="n">
+        <v>7</v>
+      </c>
       <c r="L68" t="n">
         <v>9.5</v>
       </c>
+      <c r="M68" t="n">
+        <v>7</v>
+      </c>
       <c r="P68" t="n">
         <v>1</v>
       </c>
@@ -4484,9 +4649,15 @@
       <c r="I69" t="n">
         <v>3</v>
       </c>
+      <c r="J69" t="n">
+        <v>7</v>
+      </c>
       <c r="L69" t="n">
         <v>9.5</v>
       </c>
+      <c r="M69" t="n">
+        <v>7</v>
+      </c>
       <c r="O69" t="n">
         <v>1</v>
       </c>
@@ -4541,6 +4712,9 @@
       <c r="G70" t="n">
         <v>6</v>
       </c>
+      <c r="M70" t="n">
+        <v>7</v>
+      </c>
       <c r="O70" t="n">
         <v>1</v>
       </c>
@@ -4577,11 +4751,14 @@
       <c r="I71" t="n">
         <v>5</v>
       </c>
+      <c r="J71" t="n">
+        <v>7</v>
+      </c>
       <c r="L71" t="n">
         <v>9.5</v>
       </c>
       <c r="M71" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O71" t="n">
         <v>1</v>
@@ -4643,8 +4820,11 @@
       <c r="J72" t="n">
         <v>9</v>
       </c>
+      <c r="K72" t="n">
+        <v>8</v>
+      </c>
       <c r="M72" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O72" t="n">
         <v>1</v>
@@ -4709,6 +4889,9 @@
       <c r="I73" t="n">
         <v>2</v>
       </c>
+      <c r="J73" t="n">
+        <v>7</v>
+      </c>
       <c r="L73" t="n">
         <v>11</v>
       </c>
@@ -4781,6 +4964,9 @@
       <c r="L74" t="n">
         <v>9.5</v>
       </c>
+      <c r="M74" t="n">
+        <v>7</v>
+      </c>
       <c r="O74" t="n">
         <v>1</v>
       </c>
@@ -4829,9 +5015,15 @@
       <c r="I75" t="n">
         <v>6</v>
       </c>
+      <c r="J75" t="n">
+        <v>7</v>
+      </c>
       <c r="L75" t="n">
         <v>9.5</v>
       </c>
+      <c r="M75" t="n">
+        <v>7</v>
+      </c>
       <c r="N75" t="n">
         <v>1</v>
       </c>
@@ -4955,11 +5147,14 @@
       <c r="I77" t="n">
         <v>9.5</v>
       </c>
+      <c r="J77" t="n">
+        <v>7</v>
+      </c>
       <c r="L77" t="n">
         <v>9.5</v>
       </c>
       <c r="M77" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O77" t="n">
         <v>1</v>
@@ -5009,6 +5204,9 @@
       <c r="I78" t="n">
         <v>9.5</v>
       </c>
+      <c r="J78" t="n">
+        <v>7</v>
+      </c>
       <c r="L78" t="n">
         <v>9.5</v>
       </c>
@@ -5076,11 +5274,14 @@
         <v>9.5</v>
       </c>
       <c r="J79" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L79" t="n">
         <v>9.5</v>
       </c>
+      <c r="M79" t="n">
+        <v>7</v>
+      </c>
       <c r="O79" t="n">
         <v>1</v>
       </c>
@@ -5142,7 +5343,7 @@
         <v>9.5</v>
       </c>
       <c r="M80" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O80" t="n">
         <v>1</v>
@@ -5262,7 +5463,7 @@
         <v>9</v>
       </c>
       <c r="M82" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O82" t="n">
         <v>1</v>
@@ -5426,11 +5627,14 @@
       <c r="I85" t="n">
         <v>9.5</v>
       </c>
+      <c r="J85" t="n">
+        <v>7</v>
+      </c>
       <c r="L85" t="n">
         <v>9.5</v>
       </c>
       <c r="M85" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O85" t="n">
         <v>1</v>
@@ -5498,9 +5702,15 @@
       <c r="I86" t="n">
         <v>5</v>
       </c>
+      <c r="J86" t="n">
+        <v>7</v>
+      </c>
       <c r="L86" t="n">
         <v>9.5</v>
       </c>
+      <c r="M86" t="n">
+        <v>7</v>
+      </c>
       <c r="O86" t="n">
         <v>1</v>
       </c>
@@ -5540,6 +5750,9 @@
       <c r="L87" t="n">
         <v>9.5</v>
       </c>
+      <c r="M87" t="n">
+        <v>7</v>
+      </c>
       <c r="O87" t="n">
         <v>1</v>
       </c>
@@ -5648,9 +5861,15 @@
       <c r="I89" t="n">
         <v>3</v>
       </c>
+      <c r="J89" t="n">
+        <v>7</v>
+      </c>
       <c r="L89" t="n">
         <v>9.5</v>
       </c>
+      <c r="M89" t="n">
+        <v>7</v>
+      </c>
       <c r="O89" t="n">
         <v>1</v>
       </c>
@@ -5718,7 +5937,7 @@
         <v>9.5</v>
       </c>
       <c r="M90" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O90" t="n">
         <v>1</v>
@@ -5789,11 +6008,17 @@
       <c r="I91" t="n">
         <v>9.5</v>
       </c>
+      <c r="J91" t="n">
+        <v>7</v>
+      </c>
+      <c r="K91" t="n">
+        <v>8</v>
+      </c>
       <c r="L91" t="n">
         <v>9.5</v>
       </c>
       <c r="M91" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O91" t="n">
         <v>1</v>
@@ -5975,6 +6200,9 @@
       <c r="L94" t="n">
         <v>11</v>
       </c>
+      <c r="M94" t="n">
+        <v>7</v>
+      </c>
       <c r="O94" t="n">
         <v>1</v>
       </c>
@@ -6101,6 +6329,9 @@
       <c r="I96" t="n">
         <v>8</v>
       </c>
+      <c r="J96" t="n">
+        <v>7</v>
+      </c>
       <c r="L96" t="n">
         <v>9.5</v>
       </c>
@@ -6239,6 +6470,9 @@
       <c r="I98" t="n">
         <v>9.5</v>
       </c>
+      <c r="M98" t="n">
+        <v>7</v>
+      </c>
       <c r="O98" t="n">
         <v>1</v>
       </c>
@@ -6297,7 +6531,7 @@
         <v>9.5</v>
       </c>
       <c r="M99" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="P99" t="n">
         <v>1</v>
@@ -6428,6 +6662,9 @@
       <c r="I101" t="n">
         <v>4</v>
       </c>
+      <c r="J101" t="n">
+        <v>7</v>
+      </c>
       <c r="O101" t="n">
         <v>1</v>
       </c>
@@ -6473,6 +6710,9 @@
       <c r="L102" t="n">
         <v>9.5</v>
       </c>
+      <c r="M102" t="n">
+        <v>7</v>
+      </c>
       <c r="O102" t="n">
         <v>1</v>
       </c>
@@ -6530,11 +6770,17 @@
       <c r="I103" t="n">
         <v>7</v>
       </c>
+      <c r="J103" t="n">
+        <v>7</v>
+      </c>
+      <c r="K103" t="n">
+        <v>8</v>
+      </c>
       <c r="L103" t="n">
         <v>9.5</v>
       </c>
       <c r="M103" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O103" t="n">
         <v>1</v>
@@ -6605,6 +6851,9 @@
       <c r="L104" t="n">
         <v>9.5</v>
       </c>
+      <c r="M104" t="n">
+        <v>7</v>
+      </c>
       <c r="O104" t="n">
         <v>1</v>
       </c>
@@ -6659,6 +6908,9 @@
       <c r="L105" t="n">
         <v>9.5</v>
       </c>
+      <c r="M105" t="n">
+        <v>7</v>
+      </c>
       <c r="O105" t="n">
         <v>1</v>
       </c>
@@ -6707,6 +6959,9 @@
       <c r="I106" t="n">
         <v>7</v>
       </c>
+      <c r="M106" t="n">
+        <v>7</v>
+      </c>
       <c r="O106" t="n">
         <v>1</v>
       </c>
@@ -6750,13 +7005,13 @@
         <v>8</v>
       </c>
       <c r="J107" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L107" t="n">
         <v>9.5</v>
       </c>
       <c r="M107" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="N107" t="n">
         <v>1</v>
@@ -6827,6 +7082,12 @@
       <c r="I108" t="n">
         <v>8</v>
       </c>
+      <c r="J108" t="n">
+        <v>7</v>
+      </c>
+      <c r="M108" t="n">
+        <v>7</v>
+      </c>
       <c r="O108" t="n">
         <v>1</v>
       </c>
@@ -6887,6 +7148,9 @@
       <c r="F110" t="n">
         <v>8</v>
       </c>
+      <c r="M110" t="n">
+        <v>7</v>
+      </c>
       <c r="O110" t="n">
         <v>1</v>
       </c>
@@ -6924,11 +7188,14 @@
         <v>2</v>
       </c>
       <c r="J111" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K111" t="n">
         <v>9</v>
       </c>
+      <c r="M111" t="n">
+        <v>7</v>
+      </c>
       <c r="O111" t="n">
         <v>1</v>
       </c>
@@ -6980,9 +7247,15 @@
       <c r="I112" t="n">
         <v>8</v>
       </c>
+      <c r="J112" t="n">
+        <v>7</v>
+      </c>
       <c r="L112" t="n">
         <v>9.5</v>
       </c>
+      <c r="M112" t="n">
+        <v>7</v>
+      </c>
       <c r="O112" t="n">
         <v>1</v>
       </c>
@@ -7046,6 +7319,9 @@
       <c r="I113" t="n">
         <v>2</v>
       </c>
+      <c r="J113" t="n">
+        <v>7</v>
+      </c>
       <c r="K113" t="n">
         <v>9</v>
       </c>
@@ -7053,7 +7329,7 @@
         <v>9.5</v>
       </c>
       <c r="M113" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O113" t="n">
         <v>1</v>
@@ -7119,7 +7395,7 @@
         <v>6</v>
       </c>
       <c r="J114" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K114" t="n">
         <v>9</v>
@@ -7128,7 +7404,7 @@
         <v>9.5</v>
       </c>
       <c r="M114" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O114" t="n">
         <v>1</v>
@@ -7193,6 +7469,9 @@
       <c r="G115" t="n">
         <v>8.5</v>
       </c>
+      <c r="J115" t="n">
+        <v>7</v>
+      </c>
       <c r="L115" t="n">
         <v>9.5</v>
       </c>
@@ -7251,13 +7530,13 @@
         <v>8</v>
       </c>
       <c r="J116" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L116" t="n">
         <v>9.5</v>
       </c>
       <c r="M116" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="N116" t="n">
         <v>1</v>
@@ -7332,13 +7611,13 @@
         <v>9</v>
       </c>
       <c r="K117" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L117" t="n">
         <v>9.5</v>
       </c>
       <c r="M117" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O117" t="n">
         <v>1</v>
@@ -7403,11 +7682,14 @@
       <c r="I118" t="n">
         <v>6</v>
       </c>
+      <c r="J118" t="n">
+        <v>7</v>
+      </c>
       <c r="L118" t="n">
         <v>9.5</v>
       </c>
       <c r="M118" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O118" t="n">
         <v>1</v>
@@ -7478,6 +7760,9 @@
       <c r="I119" t="n">
         <v>8</v>
       </c>
+      <c r="J119" t="n">
+        <v>7</v>
+      </c>
       <c r="L119" t="n">
         <v>9.5</v>
       </c>
@@ -7545,7 +7830,7 @@
         <v>9.5</v>
       </c>
       <c r="J120" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M120" t="n">
         <v>9.5</v>
@@ -7635,7 +7920,7 @@
         <v>9.5</v>
       </c>
       <c r="M122" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="N122" t="n">
         <v>1</v>
@@ -7703,9 +7988,15 @@
       <c r="I123" t="n">
         <v>2</v>
       </c>
+      <c r="J123" t="n">
+        <v>7</v>
+      </c>
       <c r="L123" t="n">
         <v>9.5</v>
       </c>
+      <c r="M123" t="n">
+        <v>7</v>
+      </c>
       <c r="O123" t="n">
         <v>1</v>
       </c>
@@ -7757,6 +8048,9 @@
       <c r="L124" t="n">
         <v>9.5</v>
       </c>
+      <c r="M124" t="n">
+        <v>7</v>
+      </c>
       <c r="P124" t="n">
         <v>1</v>
       </c>
@@ -7808,11 +8102,14 @@
       <c r="I125" t="n">
         <v>8</v>
       </c>
+      <c r="J125" t="n">
+        <v>7</v>
+      </c>
       <c r="L125" t="n">
         <v>9.5</v>
       </c>
       <c r="M125" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O125" t="n">
         <v>1</v>
@@ -7881,13 +8178,16 @@
         <v>5</v>
       </c>
       <c r="J126" t="n">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="K126" t="n">
+        <v>8</v>
       </c>
       <c r="L126" t="n">
         <v>9.5</v>
       </c>
       <c r="M126" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O126" t="n">
         <v>1</v>
@@ -7955,6 +8255,9 @@
       <c r="I127" t="n">
         <v>5</v>
       </c>
+      <c r="M127" t="n">
+        <v>7</v>
+      </c>
       <c r="O127" t="n">
         <v>1</v>
       </c>
@@ -8342,6 +8645,9 @@
       <c r="D138" t="n">
         <v>10</v>
       </c>
+      <c r="J138" t="n">
+        <v>7</v>
+      </c>
       <c r="L138" t="n">
         <v>9.5</v>
       </c>
@@ -8463,7 +8769,7 @@
         <v>11</v>
       </c>
       <c r="M141" t="n">
-        <v>9.5</v>
+        <v>7</v>
       </c>
       <c r="O141" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
fix(internacional): las 4 clases «no retomado» de 9.°–11.° eran falsas o parciales
La revisión crítica del bucle encontró que el método v1 de 9.°–11.° no busca
en la fila completa de la malla. Las 4 clases «no retomado» (efecto
invernadero en dos conceptos, capas de la atmósfera y usos de la energía)
aparecen en 10.° y 11.° en microhabilidades, valores o subcontenidos: pasan a
«retomado» con su cita literal verificada (decisiones delegadas, pendientes de
confirmar). README de 9.°–11.°: la atmósfera se retoma en parte y la
recomendación del equilibrio en 9.° sigue el matiz del panel. CSV para el
MINED con 175 decisiones; snapshots regenerados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/internacional/Contraste_fisica.xlsx
+++ b/internacional/Contraste_fisica.xlsx
@@ -2625,109 +2625,49 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Absorción de radiación y efecto invernadero</t>
+          <t>Materiales opacos, transparentes y translúcidos</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>no_retomado</t>
+          <t>previo</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>7</v>
-      </c>
-      <c r="E37" t="n">
-        <v>9</v>
-      </c>
-      <c r="F37" t="n">
-        <v>10.5</v>
+        <v>2</v>
       </c>
       <c r="G37" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="I37" t="n">
-        <v>10</v>
-      </c>
-      <c r="J37" t="n">
-        <v>9</v>
-      </c>
-      <c r="K37" t="n">
-        <v>9</v>
-      </c>
-      <c r="L37" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="M37" t="n">
-        <v>7</v>
-      </c>
-      <c r="N37" t="n">
-        <v>1</v>
-      </c>
-      <c r="O37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P37" t="n">
         <v>1</v>
       </c>
-      <c r="R37" t="n">
-        <v>1</v>
-      </c>
-      <c r="S37" t="n">
-        <v>1</v>
-      </c>
-      <c r="T37" t="n">
-        <v>1</v>
-      </c>
-      <c r="U37" t="n">
-        <v>1</v>
-      </c>
-      <c r="V37" t="n">
-        <v>1</v>
-      </c>
-      <c r="W37" t="n">
-        <v>1</v>
-      </c>
-      <c r="X37" t="n">
-        <v>1</v>
-      </c>
       <c r="Y37" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB37" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC37" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>La energía y sus usos</t>
+          <t>Movimiento, reposo y tipos de trayectoria</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>no_retomado</t>
+          <t>previo</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>2</v>
       </c>
-      <c r="F38" t="n">
-        <v>8</v>
+      <c r="E38" t="n">
+        <v>2</v>
       </c>
       <c r="G38" t="n">
+        <v>6</v>
+      </c>
+      <c r="I38" t="n">
         <v>2</v>
-      </c>
-      <c r="I38" t="n">
-        <v>5</v>
-      </c>
-      <c r="J38" t="n">
-        <v>7</v>
       </c>
       <c r="L38" t="n">
         <v>9.5</v>
@@ -2735,38 +2675,26 @@
       <c r="M38" t="n">
         <v>7</v>
       </c>
-      <c r="O38" t="n">
-        <v>1</v>
-      </c>
       <c r="P38" t="n">
         <v>1</v>
       </c>
-      <c r="R38" t="n">
-        <v>1</v>
-      </c>
       <c r="U38" t="n">
         <v>1</v>
       </c>
-      <c r="V38" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y38" t="n">
-        <v>1</v>
-      </c>
       <c r="Z38" t="n">
         <v>1</v>
       </c>
-      <c r="AB38" t="n">
-        <v>1</v>
-      </c>
       <c r="AC38" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD38" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Materiales opacos, transparentes y translúcidos</t>
+          <t>El sonido se produce por vibraciones</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2777,38 +2705,80 @@
       <c r="C39" t="n">
         <v>2</v>
       </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="n">
+        <v>8</v>
+      </c>
       <c r="G39" t="n">
         <v>2</v>
       </c>
-      <c r="P39" t="n">
+      <c r="I39" t="n">
+        <v>2</v>
+      </c>
+      <c r="J39" t="n">
+        <v>7</v>
+      </c>
+      <c r="L39" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="O39" t="n">
+        <v>1</v>
+      </c>
+      <c r="U39" t="n">
         <v>1</v>
       </c>
       <c r="Y39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD39" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE39" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Movimiento, reposo y tipos de trayectoria</t>
+          <t>Absorción de radiación y efecto invernadero</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>previo</t>
+          <t>retomado</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E40" t="n">
-        <v>2</v>
+        <v>9</v>
+      </c>
+      <c r="F40" t="n">
+        <v>10.5</v>
       </c>
       <c r="G40" t="n">
-        <v>6</v>
+        <v>8.5</v>
       </c>
       <c r="I40" t="n">
-        <v>2</v>
+        <v>10</v>
+      </c>
+      <c r="J40" t="n">
+        <v>9</v>
+      </c>
+      <c r="K40" t="n">
+        <v>9</v>
       </c>
       <c r="L40" t="n">
         <v>9.5</v>
@@ -2816,47 +2786,74 @@
       <c r="M40" t="n">
         <v>7</v>
       </c>
+      <c r="N40" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1</v>
+      </c>
       <c r="P40" t="n">
         <v>1</v>
       </c>
+      <c r="R40" t="n">
+        <v>1</v>
+      </c>
+      <c r="S40" t="n">
+        <v>1</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1</v>
+      </c>
       <c r="U40" t="n">
         <v>1</v>
       </c>
+      <c r="V40" t="n">
+        <v>1</v>
+      </c>
+      <c r="W40" t="n">
+        <v>1</v>
+      </c>
+      <c r="X40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>1</v>
+      </c>
       <c r="Z40" t="n">
         <v>1</v>
       </c>
+      <c r="AB40" t="n">
+        <v>1</v>
+      </c>
       <c r="AC40" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD40" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>El sonido se produce por vibraciones</t>
+          <t>Aceleración</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>previo</t>
+          <t>retomado</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2</v>
-      </c>
-      <c r="E41" t="n">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="D41" t="n">
+        <v>10</v>
       </c>
       <c r="F41" t="n">
-        <v>8</v>
+        <v>10.5</v>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>8.5</v>
       </c>
       <c r="I41" t="n">
-        <v>2</v>
+        <v>9.5</v>
       </c>
       <c r="J41" t="n">
         <v>7</v>
@@ -2864,12 +2861,27 @@
       <c r="L41" t="n">
         <v>9.5</v>
       </c>
+      <c r="M41" t="n">
+        <v>7</v>
+      </c>
       <c r="O41" t="n">
         <v>1</v>
       </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+      <c r="R41" t="n">
+        <v>1</v>
+      </c>
+      <c r="S41" t="n">
+        <v>1</v>
+      </c>
       <c r="U41" t="n">
         <v>1</v>
       </c>
+      <c r="W41" t="n">
+        <v>1</v>
+      </c>
       <c r="Y41" t="n">
         <v>1</v>
       </c>
@@ -2883,16 +2895,13 @@
         <v>1</v>
       </c>
       <c r="AD41" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE41" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Aceleración</t>
+          <t>Aceleración y fuerza centrípeta</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2909,17 +2918,8 @@
       <c r="F42" t="n">
         <v>10.5</v>
       </c>
-      <c r="G42" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="I42" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="J42" t="n">
-        <v>7</v>
-      </c>
       <c r="L42" t="n">
-        <v>9.5</v>
+        <v>11</v>
       </c>
       <c r="M42" t="n">
         <v>7</v>
@@ -2927,15 +2927,6 @@
       <c r="O42" t="n">
         <v>1</v>
       </c>
-      <c r="P42" t="n">
-        <v>1</v>
-      </c>
-      <c r="R42" t="n">
-        <v>1</v>
-      </c>
-      <c r="S42" t="n">
-        <v>1</v>
-      </c>
       <c r="U42" t="n">
         <v>1</v>
       </c>
@@ -2948,6 +2939,9 @@
       <c r="Z42" t="n">
         <v>1</v>
       </c>
+      <c r="AA42" t="n">
+        <v>1</v>
+      </c>
       <c r="AB42" t="n">
         <v>1</v>
       </c>
@@ -2955,13 +2949,16 @@
         <v>1</v>
       </c>
       <c r="AD42" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE42" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Aceleración y fuerza centrípeta</t>
+          <t>Caída libre</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2975,21 +2972,36 @@
       <c r="D43" t="n">
         <v>10</v>
       </c>
-      <c r="F43" t="n">
-        <v>10.5</v>
+      <c r="G43" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I43" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="J43" t="n">
+        <v>7</v>
       </c>
       <c r="L43" t="n">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="M43" t="n">
-        <v>7</v>
-      </c>
-      <c r="O43" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
+      <c r="R43" t="n">
+        <v>1</v>
+      </c>
+      <c r="S43" t="n">
         <v>1</v>
       </c>
       <c r="U43" t="n">
         <v>1</v>
       </c>
+      <c r="V43" t="n">
+        <v>1</v>
+      </c>
       <c r="W43" t="n">
         <v>1</v>
       </c>
@@ -2997,12 +3009,6 @@
         <v>1</v>
       </c>
       <c r="Z43" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA43" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB43" t="n">
         <v>1</v>
       </c>
       <c r="AC43" t="n">
@@ -3018,7 +3024,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Caída libre</t>
+          <t>Calentamiento y enfriamiento</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3027,16 +3033,22 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
         <v>10</v>
       </c>
+      <c r="E44" t="n">
+        <v>2</v>
+      </c>
+      <c r="F44" t="n">
+        <v>8</v>
+      </c>
       <c r="G44" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="I44" t="n">
-        <v>9.5</v>
+        <v>2</v>
       </c>
       <c r="J44" t="n">
         <v>7</v>
@@ -3045,23 +3057,17 @@
         <v>9.5</v>
       </c>
       <c r="M44" t="n">
-        <v>9.5</v>
+        <v>7</v>
+      </c>
+      <c r="O44" t="n">
+        <v>1</v>
       </c>
       <c r="P44" t="n">
         <v>1</v>
       </c>
-      <c r="R44" t="n">
-        <v>1</v>
-      </c>
-      <c r="S44" t="n">
-        <v>1</v>
-      </c>
       <c r="U44" t="n">
         <v>1</v>
       </c>
-      <c r="V44" t="n">
-        <v>1</v>
-      </c>
       <c r="W44" t="n">
         <v>1</v>
       </c>
@@ -3071,20 +3077,17 @@
       <c r="Z44" t="n">
         <v>1</v>
       </c>
-      <c r="AC44" t="n">
+      <c r="AB44" t="n">
         <v>1</v>
       </c>
       <c r="AD44" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE44" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Calentamiento y enfriamiento</t>
+          <t>Calor como energía en tránsito</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3093,13 +3096,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
-      </c>
-      <c r="E45" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F45" t="n">
         <v>8</v>
@@ -3108,7 +3108,7 @@
         <v>6</v>
       </c>
       <c r="I45" t="n">
-        <v>2</v>
+        <v>9.5</v>
       </c>
       <c r="J45" t="n">
         <v>7</v>
@@ -3125,7 +3125,13 @@
       <c r="P45" t="n">
         <v>1</v>
       </c>
+      <c r="R45" t="n">
+        <v>1</v>
+      </c>
       <c r="U45" t="n">
+        <v>1</v>
+      </c>
+      <c r="V45" t="n">
         <v>1</v>
       </c>
       <c r="W45" t="n">
@@ -3147,7 +3153,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Calor como energía en tránsito</t>
+          <t>Cambios de estado</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3156,7 +3162,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D46" t="n">
         <v>9</v>
@@ -3168,7 +3174,7 @@
         <v>6</v>
       </c>
       <c r="I46" t="n">
-        <v>9.5</v>
+        <v>3</v>
       </c>
       <c r="J46" t="n">
         <v>7</v>
@@ -3197,13 +3203,22 @@
       <c r="W46" t="n">
         <v>1</v>
       </c>
+      <c r="X46" t="n">
+        <v>1</v>
+      </c>
       <c r="Y46" t="n">
         <v>1</v>
       </c>
       <c r="Z46" t="n">
         <v>1</v>
       </c>
+      <c r="AA46" t="n">
+        <v>1</v>
+      </c>
       <c r="AB46" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC46" t="n">
         <v>1</v>
       </c>
       <c r="AD46" t="n">
@@ -3213,7 +3228,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Cambios de estado</t>
+          <t>Campo magnético y magnetismo terrestre</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -3222,7 +3237,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D47" t="n">
         <v>9</v>
@@ -3234,7 +3249,7 @@
         <v>6</v>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="J47" t="n">
         <v>7</v>
@@ -3254,6 +3269,9 @@
       <c r="R47" t="n">
         <v>1</v>
       </c>
+      <c r="S47" t="n">
+        <v>1</v>
+      </c>
       <c r="U47" t="n">
         <v>1</v>
       </c>
@@ -3263,9 +3281,6 @@
       <c r="W47" t="n">
         <v>1</v>
       </c>
-      <c r="X47" t="n">
-        <v>1</v>
-      </c>
       <c r="Y47" t="n">
         <v>1</v>
       </c>
@@ -3282,13 +3297,16 @@
         <v>1</v>
       </c>
       <c r="AD47" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE47" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Campo magnético y magnetismo terrestre</t>
+          <t>Capacidad calorífica y calor específico</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -3297,7 +3315,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D48" t="n">
         <v>9</v>
@@ -3306,17 +3324,11 @@
         <v>8</v>
       </c>
       <c r="G48" t="n">
-        <v>6</v>
-      </c>
-      <c r="I48" t="n">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="J48" t="n">
         <v>7</v>
       </c>
-      <c r="L48" t="n">
-        <v>9.5</v>
-      </c>
       <c r="M48" t="n">
         <v>7</v>
       </c>
@@ -3326,18 +3338,6 @@
       <c r="P48" t="n">
         <v>1</v>
       </c>
-      <c r="R48" t="n">
-        <v>1</v>
-      </c>
-      <c r="S48" t="n">
-        <v>1</v>
-      </c>
-      <c r="U48" t="n">
-        <v>1</v>
-      </c>
-      <c r="V48" t="n">
-        <v>1</v>
-      </c>
       <c r="W48" t="n">
         <v>1</v>
       </c>
@@ -3347,9 +3347,6 @@
       <c r="Z48" t="n">
         <v>1</v>
       </c>
-      <c r="AA48" t="n">
-        <v>1</v>
-      </c>
       <c r="AB48" t="n">
         <v>1</v>
       </c>
@@ -3357,16 +3354,13 @@
         <v>1</v>
       </c>
       <c r="AD48" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE48" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Capacidad calorífica y calor específico</t>
+          <t>Carga eléctrica y electrización</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3375,7 +3369,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D49" t="n">
         <v>9</v>
@@ -3384,11 +3378,20 @@
         <v>8</v>
       </c>
       <c r="G49" t="n">
-        <v>8.5</v>
+        <v>6</v>
+      </c>
+      <c r="I49" t="n">
+        <v>7</v>
       </c>
       <c r="J49" t="n">
         <v>7</v>
       </c>
+      <c r="K49" t="n">
+        <v>8</v>
+      </c>
+      <c r="L49" t="n">
+        <v>9.5</v>
+      </c>
       <c r="M49" t="n">
         <v>7</v>
       </c>
@@ -3398,6 +3401,12 @@
       <c r="P49" t="n">
         <v>1</v>
       </c>
+      <c r="U49" t="n">
+        <v>1</v>
+      </c>
+      <c r="V49" t="n">
+        <v>1</v>
+      </c>
       <c r="W49" t="n">
         <v>1</v>
       </c>
@@ -3407,20 +3416,23 @@
       <c r="Z49" t="n">
         <v>1</v>
       </c>
+      <c r="AA49" t="n">
+        <v>1</v>
+      </c>
       <c r="AB49" t="n">
         <v>1</v>
       </c>
-      <c r="AC49" t="n">
-        <v>1</v>
-      </c>
       <c r="AD49" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE49" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Carga eléctrica y electrización</t>
+          <t>Circuito eléctrico simple</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -3429,19 +3441,22 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D50" t="n">
         <v>9</v>
       </c>
+      <c r="E50" t="n">
+        <v>5</v>
+      </c>
       <c r="F50" t="n">
         <v>8</v>
       </c>
       <c r="G50" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I50" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J50" t="n">
         <v>7</v>
@@ -3464,9 +3479,6 @@
       <c r="U50" t="n">
         <v>1</v>
       </c>
-      <c r="V50" t="n">
-        <v>1</v>
-      </c>
       <c r="W50" t="n">
         <v>1</v>
       </c>
@@ -3476,10 +3488,10 @@
       <c r="Z50" t="n">
         <v>1</v>
       </c>
-      <c r="AA50" t="n">
-        <v>1</v>
-      </c>
       <c r="AB50" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC50" t="n">
         <v>1</v>
       </c>
       <c r="AD50" t="n">
@@ -3492,7 +3504,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Circuito eléctrico simple</t>
+          <t>Circuitos en serie y en paralelo</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3501,22 +3513,19 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D51" t="n">
         <v>9</v>
       </c>
-      <c r="E51" t="n">
-        <v>5</v>
-      </c>
       <c r="F51" t="n">
         <v>8</v>
       </c>
       <c r="G51" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J51" t="n">
         <v>7</v>
@@ -3527,9 +3536,6 @@
       <c r="L51" t="n">
         <v>9.5</v>
       </c>
-      <c r="M51" t="n">
-        <v>7</v>
-      </c>
       <c r="O51" t="n">
         <v>1</v>
       </c>
@@ -3549,9 +3555,6 @@
         <v>1</v>
       </c>
       <c r="AB51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC51" t="n">
         <v>1</v>
       </c>
       <c r="AD51" t="n">
@@ -3564,7 +3567,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Circuitos en serie y en paralelo</t>
+          <t>Colisiones elásticas e inelásticas</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3573,35 +3576,26 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D52" t="n">
+        <v>10</v>
+      </c>
+      <c r="G52" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="J52" t="n">
         <v>9</v>
       </c>
-      <c r="F52" t="n">
-        <v>8</v>
-      </c>
-      <c r="G52" t="n">
-        <v>6</v>
-      </c>
-      <c r="I52" t="n">
-        <v>3</v>
-      </c>
-      <c r="J52" t="n">
-        <v>7</v>
-      </c>
-      <c r="K52" t="n">
-        <v>8</v>
-      </c>
       <c r="L52" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="O52" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="P52" t="n">
         <v>1</v>
       </c>
+      <c r="S52" t="n">
+        <v>1</v>
+      </c>
       <c r="U52" t="n">
         <v>1</v>
       </c>
@@ -3614,7 +3608,13 @@
       <c r="Z52" t="n">
         <v>1</v>
       </c>
+      <c r="AA52" t="n">
+        <v>1</v>
+      </c>
       <c r="AB52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC52" t="n">
         <v>1</v>
       </c>
       <c r="AD52" t="n">
@@ -3627,7 +3627,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Colisiones elásticas e inelásticas</t>
+          <t>Color y dispersión de la luz</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3636,30 +3636,33 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D53" t="n">
         <v>10</v>
       </c>
+      <c r="F53" t="n">
+        <v>8</v>
+      </c>
       <c r="G53" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="J53" t="n">
+        <v>7</v>
+      </c>
+      <c r="K53" t="n">
         <v>9</v>
       </c>
-      <c r="L53" t="n">
-        <v>11</v>
-      </c>
-      <c r="P53" t="n">
+      <c r="M53" t="n">
+        <v>7</v>
+      </c>
+      <c r="O53" t="n">
         <v>1</v>
       </c>
       <c r="S53" t="n">
         <v>1</v>
       </c>
-      <c r="U53" t="n">
-        <v>1</v>
-      </c>
-      <c r="W53" t="n">
+      <c r="T53" t="n">
         <v>1</v>
       </c>
       <c r="Y53" t="n">
@@ -3668,26 +3671,17 @@
       <c r="Z53" t="n">
         <v>1</v>
       </c>
-      <c r="AA53" t="n">
-        <v>1</v>
-      </c>
       <c r="AB53" t="n">
         <v>1</v>
       </c>
       <c r="AC53" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD53" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE53" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Color y dispersión de la luz</t>
+          <t>Conductores y aislantes eléctricos</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3696,22 +3690,31 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D54" t="n">
         <v>10</v>
       </c>
+      <c r="E54" t="n">
+        <v>5</v>
+      </c>
       <c r="F54" t="n">
         <v>8</v>
       </c>
       <c r="G54" t="n">
-        <v>6</v>
+        <v>2</v>
+      </c>
+      <c r="I54" t="n">
+        <v>2</v>
       </c>
       <c r="J54" t="n">
         <v>7</v>
       </c>
       <c r="K54" t="n">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="L54" t="n">
+        <v>9.5</v>
       </c>
       <c r="M54" t="n">
         <v>7</v>
@@ -3719,10 +3722,16 @@
       <c r="O54" t="n">
         <v>1</v>
       </c>
+      <c r="R54" t="n">
+        <v>1</v>
+      </c>
       <c r="S54" t="n">
         <v>1</v>
       </c>
-      <c r="T54" t="n">
+      <c r="U54" t="n">
+        <v>1</v>
+      </c>
+      <c r="X54" t="n">
         <v>1</v>
       </c>
       <c r="Y54" t="n">
@@ -3734,14 +3743,14 @@
       <c r="AB54" t="n">
         <v>1</v>
       </c>
-      <c r="AC54" t="n">
+      <c r="AD54" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Conductores y aislantes eléctricos</t>
+          <t>Conservación de la energía mecánica</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3750,28 +3759,22 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D55" t="n">
-        <v>10</v>
-      </c>
-      <c r="E55" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F55" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G55" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I55" t="n">
         <v>8</v>
       </c>
-      <c r="G55" t="n">
-        <v>2</v>
-      </c>
-      <c r="I55" t="n">
-        <v>2</v>
-      </c>
       <c r="J55" t="n">
         <v>7</v>
-      </c>
-      <c r="K55" t="n">
-        <v>8</v>
       </c>
       <c r="L55" t="n">
         <v>9.5</v>
@@ -3782,35 +3785,41 @@
       <c r="O55" t="n">
         <v>1</v>
       </c>
+      <c r="P55" t="n">
+        <v>1</v>
+      </c>
       <c r="R55" t="n">
         <v>1</v>
       </c>
-      <c r="S55" t="n">
-        <v>1</v>
-      </c>
       <c r="U55" t="n">
         <v>1</v>
       </c>
-      <c r="X55" t="n">
-        <v>1</v>
-      </c>
       <c r="Y55" t="n">
         <v>1</v>
       </c>
       <c r="Z55" t="n">
         <v>1</v>
       </c>
+      <c r="AA55" t="n">
+        <v>1</v>
+      </c>
       <c r="AB55" t="n">
         <v>1</v>
       </c>
+      <c r="AC55" t="n">
+        <v>1</v>
+      </c>
       <c r="AD55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE55" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Conservación de la energía mecánica</t>
+          <t>Conservación del momento lineal</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3819,10 +3828,10 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D56" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F56" t="n">
         <v>10.5</v>
@@ -3830,17 +3839,8 @@
       <c r="G56" t="n">
         <v>8.5</v>
       </c>
-      <c r="I56" t="n">
-        <v>8</v>
-      </c>
-      <c r="J56" t="n">
-        <v>7</v>
-      </c>
       <c r="L56" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="M56" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O56" t="n">
         <v>1</v>
@@ -3848,10 +3848,10 @@
       <c r="P56" t="n">
         <v>1</v>
       </c>
-      <c r="R56" t="n">
-        <v>1</v>
-      </c>
       <c r="U56" t="n">
+        <v>1</v>
+      </c>
+      <c r="W56" t="n">
         <v>1</v>
       </c>
       <c r="Y56" t="n">
@@ -3879,7 +3879,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Conservación del momento lineal</t>
+          <t>Corriente, voltaje y resistencia</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3888,19 +3888,31 @@
         </is>
       </c>
       <c r="C57" t="n">
+        <v>6</v>
+      </c>
+      <c r="D57" t="n">
+        <v>9</v>
+      </c>
+      <c r="F57" t="n">
         <v>8</v>
       </c>
-      <c r="D57" t="n">
-        <v>10</v>
-      </c>
-      <c r="F57" t="n">
-        <v>10.5</v>
-      </c>
       <c r="G57" t="n">
-        <v>8.5</v>
+        <v>4</v>
+      </c>
+      <c r="I57" t="n">
+        <v>3</v>
+      </c>
+      <c r="J57" t="n">
+        <v>7</v>
+      </c>
+      <c r="K57" t="n">
+        <v>8</v>
       </c>
       <c r="L57" t="n">
-        <v>11</v>
+        <v>9.5</v>
+      </c>
+      <c r="M57" t="n">
+        <v>7</v>
       </c>
       <c r="O57" t="n">
         <v>1</v>
@@ -3908,7 +3920,13 @@
       <c r="P57" t="n">
         <v>1</v>
       </c>
+      <c r="R57" t="n">
+        <v>1</v>
+      </c>
       <c r="U57" t="n">
+        <v>1</v>
+      </c>
+      <c r="V57" t="n">
         <v>1</v>
       </c>
       <c r="W57" t="n">
@@ -3939,7 +3957,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Corriente, voltaje y resistencia</t>
+          <t>Expansión del universo y Big Bang</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3948,19 +3966,19 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D58" t="n">
+        <v>11</v>
+      </c>
+      <c r="E58" t="n">
         <v>9</v>
       </c>
       <c r="F58" t="n">
-        <v>8</v>
-      </c>
-      <c r="G58" t="n">
-        <v>4</v>
+        <v>10.5</v>
       </c>
       <c r="I58" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J58" t="n">
         <v>7</v>
@@ -3968,22 +3986,19 @@
       <c r="K58" t="n">
         <v>8</v>
       </c>
-      <c r="L58" t="n">
+      <c r="M58" t="n">
         <v>9.5</v>
       </c>
-      <c r="M58" t="n">
-        <v>7</v>
+      <c r="N58" t="n">
+        <v>1</v>
       </c>
       <c r="O58" t="n">
         <v>1</v>
       </c>
-      <c r="P58" t="n">
-        <v>1</v>
-      </c>
       <c r="R58" t="n">
         <v>1</v>
       </c>
-      <c r="U58" t="n">
+      <c r="S58" t="n">
         <v>1</v>
       </c>
       <c r="V58" t="n">
@@ -3992,6 +4007,9 @@
       <c r="W58" t="n">
         <v>1</v>
       </c>
+      <c r="X58" t="n">
+        <v>1</v>
+      </c>
       <c r="Y58" t="n">
         <v>1</v>
       </c>
@@ -4008,16 +4026,13 @@
         <v>1</v>
       </c>
       <c r="AD58" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE58" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Expansión del universo y Big Bang</t>
+          <t>Densidad</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4026,63 +4041,42 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D59" t="n">
-        <v>11</v>
-      </c>
-      <c r="E59" t="n">
         <v>9</v>
       </c>
       <c r="F59" t="n">
-        <v>10.5</v>
+        <v>8</v>
+      </c>
+      <c r="G59" t="n">
+        <v>6</v>
       </c>
       <c r="I59" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J59" t="n">
         <v>7</v>
       </c>
-      <c r="K59" t="n">
-        <v>8</v>
+      <c r="L59" t="n">
+        <v>9.5</v>
       </c>
       <c r="M59" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="N59" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="O59" t="n">
         <v>1</v>
       </c>
-      <c r="R59" t="n">
-        <v>1</v>
-      </c>
-      <c r="S59" t="n">
-        <v>1</v>
-      </c>
-      <c r="V59" t="n">
-        <v>1</v>
-      </c>
-      <c r="W59" t="n">
-        <v>1</v>
-      </c>
-      <c r="X59" t="n">
+      <c r="P59" t="n">
+        <v>1</v>
+      </c>
+      <c r="U59" t="n">
         <v>1</v>
       </c>
       <c r="Y59" t="n">
         <v>1</v>
       </c>
       <c r="Z59" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA59" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB59" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC59" t="n">
         <v>1</v>
       </c>
       <c r="AD59" t="n">
@@ -4092,7 +4086,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Densidad</t>
+          <t>Dilatación térmica</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4101,10 +4095,10 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D60" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F60" t="n">
         <v>8</v>
@@ -4113,7 +4107,7 @@
         <v>6</v>
       </c>
       <c r="I60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J60" t="n">
         <v>7</v>
@@ -4127,26 +4121,17 @@
       <c r="O60" t="n">
         <v>1</v>
       </c>
-      <c r="P60" t="n">
-        <v>1</v>
-      </c>
       <c r="U60" t="n">
         <v>1</v>
       </c>
-      <c r="Y60" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z60" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD60" t="n">
+      <c r="AB60" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Dilatación térmica</t>
+          <t>Dinámica y energía de rotación</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4155,43 +4140,19 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D61" t="n">
         <v>10</v>
       </c>
-      <c r="F61" t="n">
-        <v>8</v>
-      </c>
-      <c r="G61" t="n">
-        <v>6</v>
-      </c>
-      <c r="I61" t="n">
-        <v>3</v>
-      </c>
-      <c r="J61" t="n">
-        <v>7</v>
-      </c>
-      <c r="L61" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="M61" t="n">
-        <v>7</v>
-      </c>
-      <c r="O61" t="n">
-        <v>1</v>
-      </c>
-      <c r="U61" t="n">
-        <v>1</v>
-      </c>
-      <c r="AB61" t="n">
+      <c r="Z61" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Dinámica y energía de rotación</t>
+          <t>Disipación de energía y eficiencia</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4200,19 +4161,76 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
-        <v>10</v>
+        <v>9</v>
+      </c>
+      <c r="E62" t="n">
+        <v>8</v>
+      </c>
+      <c r="F62" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="G62" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I62" t="n">
+        <v>8</v>
+      </c>
+      <c r="J62" t="n">
+        <v>7</v>
+      </c>
+      <c r="K62" t="n">
+        <v>8</v>
+      </c>
+      <c r="L62" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="M62" t="n">
+        <v>7</v>
+      </c>
+      <c r="O62" t="n">
+        <v>1</v>
+      </c>
+      <c r="P62" t="n">
+        <v>1</v>
+      </c>
+      <c r="R62" t="n">
+        <v>1</v>
+      </c>
+      <c r="S62" t="n">
+        <v>1</v>
+      </c>
+      <c r="U62" t="n">
+        <v>1</v>
+      </c>
+      <c r="V62" t="n">
+        <v>1</v>
+      </c>
+      <c r="W62" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>1</v>
       </c>
       <c r="Z62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AB62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AD62" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Disipación de energía y eficiencia</t>
+          <t>Electroimanes y efecto magnético de la corriente</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -4221,28 +4239,22 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D63" t="n">
         <v>9</v>
       </c>
-      <c r="E63" t="n">
+      <c r="F63" t="n">
         <v>8</v>
       </c>
-      <c r="F63" t="n">
-        <v>10.5</v>
-      </c>
       <c r="G63" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="I63" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J63" t="n">
         <v>7</v>
-      </c>
-      <c r="K63" t="n">
-        <v>8</v>
       </c>
       <c r="L63" t="n">
         <v>9.5</v>
@@ -4256,27 +4268,24 @@
       <c r="P63" t="n">
         <v>1</v>
       </c>
-      <c r="R63" t="n">
-        <v>1</v>
-      </c>
-      <c r="S63" t="n">
-        <v>1</v>
-      </c>
       <c r="U63" t="n">
         <v>1</v>
       </c>
-      <c r="V63" t="n">
-        <v>1</v>
-      </c>
       <c r="W63" t="n">
         <v>1</v>
       </c>
+      <c r="X63" t="n">
+        <v>1</v>
+      </c>
       <c r="Y63" t="n">
         <v>1</v>
       </c>
       <c r="Z63" t="n">
         <v>1</v>
       </c>
+      <c r="AA63" t="n">
+        <v>1</v>
+      </c>
       <c r="AB63" t="n">
         <v>1</v>
       </c>
@@ -4284,13 +4293,16 @@
         <v>1</v>
       </c>
       <c r="AD63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE63" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Electroimanes y efecto magnético de la corriente</t>
+          <t>Energía cinética</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4299,19 +4311,19 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
-      </c>
-      <c r="F64" t="n">
+        <v>10</v>
+      </c>
+      <c r="E64" t="n">
+        <v>7</v>
+      </c>
+      <c r="G64" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I64" t="n">
         <v>8</v>
-      </c>
-      <c r="G64" t="n">
-        <v>6</v>
-      </c>
-      <c r="I64" t="n">
-        <v>4</v>
       </c>
       <c r="J64" t="n">
         <v>7</v>
@@ -4322,19 +4334,22 @@
       <c r="M64" t="n">
         <v>7</v>
       </c>
-      <c r="O64" t="n">
-        <v>1</v>
-      </c>
       <c r="P64" t="n">
         <v>1</v>
       </c>
+      <c r="R64" t="n">
+        <v>1</v>
+      </c>
+      <c r="S64" t="n">
+        <v>1</v>
+      </c>
       <c r="U64" t="n">
         <v>1</v>
       </c>
+      <c r="V64" t="n">
+        <v>1</v>
+      </c>
       <c r="W64" t="n">
-        <v>1</v>
-      </c>
-      <c r="X64" t="n">
         <v>1</v>
       </c>
       <c r="Y64" t="n">
@@ -4362,7 +4377,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Energía cinética</t>
+          <t>Energía potencial gravitatoria y elástica</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4380,7 +4395,7 @@
         <v>7</v>
       </c>
       <c r="G65" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="I65" t="n">
         <v>8</v>
@@ -4400,15 +4415,9 @@
       <c r="R65" t="n">
         <v>1</v>
       </c>
-      <c r="S65" t="n">
-        <v>1</v>
-      </c>
       <c r="U65" t="n">
         <v>1</v>
       </c>
-      <c r="V65" t="n">
-        <v>1</v>
-      </c>
       <c r="W65" t="n">
         <v>1</v>
       </c>
@@ -4416,9 +4425,6 @@
         <v>1</v>
       </c>
       <c r="Z65" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA65" t="n">
         <v>1</v>
       </c>
       <c r="AB65" t="n">
@@ -4437,7 +4443,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Energía potencial gravitatoria y elástica</t>
+          <t>La energía y sus usos</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4446,19 +4452,16 @@
         </is>
       </c>
       <c r="C66" t="n">
+        <v>2</v>
+      </c>
+      <c r="F66" t="n">
+        <v>8</v>
+      </c>
+      <c r="G66" t="n">
+        <v>2</v>
+      </c>
+      <c r="I66" t="n">
         <v>5</v>
-      </c>
-      <c r="D66" t="n">
-        <v>10</v>
-      </c>
-      <c r="E66" t="n">
-        <v>7</v>
-      </c>
-      <c r="G66" t="n">
-        <v>6</v>
-      </c>
-      <c r="I66" t="n">
-        <v>8</v>
       </c>
       <c r="J66" t="n">
         <v>7</v>
@@ -4469,6 +4472,9 @@
       <c r="M66" t="n">
         <v>7</v>
       </c>
+      <c r="O66" t="n">
+        <v>1</v>
+      </c>
       <c r="P66" t="n">
         <v>1</v>
       </c>
@@ -4478,7 +4484,7 @@
       <c r="U66" t="n">
         <v>1</v>
       </c>
-      <c r="W66" t="n">
+      <c r="V66" t="n">
         <v>1</v>
       </c>
       <c r="Y66" t="n">
@@ -4491,12 +4497,6 @@
         <v>1</v>
       </c>
       <c r="AC66" t="n">
-        <v>1</v>
-      </c>
-      <c r="AD66" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE66" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>